<commit_message>
fix(frontend): align upload hints and file pickers with accepted formats
Design upload hints said PNG/JPG, but the server only accepts PNG and SVG
(UploadDesignFileRequest). Update the id/en hint text and the file input
accept attribute on product detail, customize and bulk order, and adjust
the matching QC checklist points.
</commit_message>
<xml_diff>
--- a/Required Document/QC_Manual_Testing_Checklist.xlsx
+++ b/Required Document/QC_Manual_Testing_Checklist.xlsx
@@ -7692,7 +7692,7 @@
       <c r="E78" s="22" t="n"/>
       <c r="F78" s="27" t="inlineStr">
         <is>
-          <t>Area upload "Upload Desain Sendiri (opsional)": file PNG ≤ 20MB (UI menyebut PNG/JPG, padahal server hanya menerima PNG &amp; SVG — uji JPG &amp; SVG, catat ketidaksesuaian) berhasil, status berubah "File terunggah", dapat diganti</t>
+          <t>Area upload "Upload Desain Sendiri (opsional)": file PNG/SVG ≤ 20MB (teks UI menyebut PNG/SVG; file JPG ditolak dengan pesan jelas) berhasil, status berubah "File terunggah", dapat diganti</t>
         </is>
       </c>
       <c r="G78" s="24" t="inlineStr">
@@ -10605,7 +10605,7 @@
       </c>
       <c r="H20" s="27" t="n"/>
     </row>
-    <row r="21" ht="54" customHeight="1">
+    <row r="21" ht="40.5" customHeight="1">
       <c r="A21" s="24" t="n">
         <v>20</v>
       </c>
@@ -10615,7 +10615,7 @@
       <c r="E21" s="22" t="n"/>
       <c r="F21" s="27" t="inlineStr">
         <is>
-          <t>Mode Custom: upload desain sendiri (PNG ≤ 20MB (UI menyebut PNG/JPG, padahal server hanya menerima PNG &amp; SVG — uji JPG &amp; SVG, catat ketidaksesuaian)) berhasil; file salah format/terlalu besar ditolak</t>
+          <t>Mode Custom: upload desain sendiri (PNG/SVG ≤ 20MB (teks UI menyebut PNG/SVG; file JPG ditolak dengan pesan jelas)) berhasil; file salah format/terlalu besar ditolak</t>
         </is>
       </c>
       <c r="G21" s="24" t="inlineStr">

</xml_diff>